<commit_message>
Update dashboard and demo video assets
</commit_message>
<xml_diff>
--- a/TeacherTraining/templates/attendance-template.xlsx
+++ b/TeacherTraining/templates/attendance-template.xlsx
@@ -55,7 +55,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-11</t>
+          <t xml:space="preserve">2026-10-16</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -82,7 +82,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-11</t>
+          <t xml:space="preserve">2026-10-16</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">

</xml_diff>